<commit_message>
update version number 382362544cba4d58ccfe1ef59e2a91fc72d24a75
</commit_message>
<xml_diff>
--- a/nr-prepare-ballot-release/ig/CodeSystem-fr-additional-action-relationship-type.xlsx
+++ b/nr-prepare-ballot-release/ig/CodeSystem-fr-additional-action-relationship-type.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0-ballot</t>
+    <t>1.1.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-06T13:17:36+00:00</t>
+    <t>2026-05-06T13:22:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>